<commit_message>
Added currency symbols for clarity
</commit_message>
<xml_diff>
--- a/Tech-Employee-Workforce-Analysis/Tech_Employee_Survey_Cleaned.xlsx
+++ b/Tech-Employee-Workforce-Analysis/Tech_Employee_Survey_Cleaned.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\Data cleaning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C31B860-AD47-4A63-BE85-6BF7C98B8899}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB8175F8-6EE7-4CD1-BF95-EBA6301BFA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="10920" activeTab="1" xr2:uid="{3103E588-A9CD-4437-B183-5CFC39FC6AC1}"/>
   </bookViews>
@@ -21,13 +21,13 @@
   </sheets>
   <calcPr calcId="181029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId6"/>
+    <pivotCache cacheId="19" r:id="rId6"/>
   </pivotCaches>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="159">
   <si>
     <t>Employee_ID</t>
   </si>
@@ -349,29 +349,6 @@
   </si>
   <si>
     <t>A fully cleaned and analysis-ready dataset, supported by a clear dashboard and documented methodology, enabling reliable insights and decision-making.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">NOTE: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>The charts excludes missing/unknown values for clarity.</t>
-    </r>
   </si>
   <si>
     <t>TECH EMPLOYEE SURVEY DATA CLEANING AND ANALYSIS PROJECT</t>
@@ -752,13 +729,23 @@
   <si>
     <t>3. Average Number of year of Experience</t>
   </si>
+  <si>
+    <t>• The charts excludes missing/unknown values for clarity.</t>
+  </si>
+  <si>
+    <t>• Currency not specified in source data; values presented for analytical purposes.</t>
+  </si>
+  <si>
+    <t>NOTE:</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="25" x14ac:knownFonts="1">
@@ -1287,7 +1274,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1308,6 +1295,9 @@
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="44" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1365,7 +1355,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="27">
+  <dxfs count="28">
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
@@ -1415,7 +1405,7 @@
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="35" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="34" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -1433,13 +1423,16 @@
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="35" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
+      <numFmt numFmtId="34" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="35" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
       <fill>
@@ -1458,8 +1451,8 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="PivotTable Style 1" table="0" count="2" xr9:uid="{85DBF63A-314B-42E2-B3FD-8382E1D367D5}">
-      <tableStyleElement type="headerRow" dxfId="26"/>
-      <tableStyleElement type="totalRow" dxfId="25"/>
+      <tableStyleElement type="headerRow" dxfId="27"/>
+      <tableStyleElement type="totalRow" dxfId="26"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -1673,7 +1666,7 @@
             <c:numRef>
               <c:f>'02_SUMMARY'!$B$7:$B$9</c:f>
               <c:numCache>
-                <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
+                <c:formatCode>_("$"* #,##0.00_);_("$"* \(#,##0.00\);_("$"* "-"??_);_(@_)</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>77200</c:v>
@@ -1756,7 +1749,7 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:numFmt formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)" sourceLinked="1"/>
+        <c:numFmt formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1967,25 +1960,29 @@
         <c:dLbl>
           <c:idx val="0"/>
           <c:spPr>
-            <a:noFill/>
+            <a:solidFill>
+              <a:sysClr val="window" lastClr="FFFFFF"/>
+            </a:solidFill>
             <a:ln>
-              <a:noFill/>
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="25000"/>
+                  <a:lumOff val="75000"/>
+                </a:sysClr>
+              </a:solidFill>
             </a:ln>
             <a:effectLst/>
           </c:spPr>
           <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
               <a:spAutoFit/>
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="75000"/>
-                      <a:lumOff val="25000"/>
-                    </a:schemeClr>
+                    <a:schemeClr val="tx1"/>
                   </a:solidFill>
                   <a:latin typeface="+mn-lt"/>
                   <a:ea typeface="+mn-ea"/>
@@ -1995,14 +1992,25 @@
               <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
+          <c:dLblPos val="outEnd"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
           <c:showCatName val="0"/>
           <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
+          <c:showPercent val="1"/>
           <c:showBubbleSize val="0"/>
           <c:extLst>
-            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+              <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                <a:prstGeom prst="wedgeRectCallout">
+                  <a:avLst/>
+                </a:prstGeom>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+              </c15:spPr>
+            </c:ext>
           </c:extLst>
         </c:dLbl>
       </c:pivotFmt>
@@ -2101,6 +2109,62 @@
               </c:ext>
             </c:extLst>
           </c:dPt>
+          <c:dLbls>
+            <c:spPr>
+              <a:solidFill>
+                <a:sysClr val="window" lastClr="FFFFFF"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000">
+                    <a:lumMod val="25000"/>
+                    <a:lumOff val="75000"/>
+                  </a:sysClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="1"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <a:prstGeom prst="wedgeRectCallout">
+                    <a:avLst/>
+                  </a:prstGeom>
+                  <a:noFill/>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                </c15:spPr>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:strRef>
               <c:f>'02_SUMMARY'!$A$15:$A$17</c:f>
@@ -2143,7 +2207,7 @@
           <c:showSerName val="0"/>
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
-          <c:showLeaderLines val="1"/>
+          <c:showLeaderLines val="0"/>
         </c:dLbls>
         <c:firstSliceAng val="0"/>
       </c:pieChart>
@@ -2528,6 +2592,8 @@
         <c:axId val="1283566944"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:max val="20"/>
+          <c:min val="0"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -2562,6 +2628,7 @@
         <c:crossAx val="1283565024"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
+        <c:majorUnit val="4"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -4845,15 +4912,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>9923</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>33338</xdr:rowOff>
+      <xdr:colOff>9922</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>195263</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>3153103</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>153276</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>3829050</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4880,16 +4947,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>3306488</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>4038600</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>22157</xdr:rowOff>
+      <xdr:rowOff>3109</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>600329</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>149554</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>6838949</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>95251</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4916,16 +4983,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>951450</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>71539</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>2352676</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>1248101</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>10948</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>5553076</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>95251</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4954,7 +5021,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="DELL" refreshedDate="46114.465139236112" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="25" xr:uid="{CF44B33C-0C99-4D95-8E06-0CFEC841BFCB}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="DELL" refreshedDate="46132.684413657407" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="25" xr:uid="{CF44B33C-0C99-4D95-8E06-0CFEC841BFCB}">
   <cacheSource type="worksheet">
     <worksheetSource name="Table2"/>
   </cacheSource>
@@ -4975,7 +5042,7 @@
         <s v="N/A"/>
       </sharedItems>
     </cacheField>
-    <cacheField name="Salary" numFmtId="43">
+    <cacheField name="Salary" numFmtId="44">
       <sharedItems containsBlank="1" containsMixedTypes="1" containsNumber="1" containsInteger="1" minValue="50000" maxValue="120000"/>
     </cacheField>
     <cacheField name="Years_of_Experience" numFmtId="1">
@@ -5316,101 +5383,17 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E9C9B4EC-AE72-4272-AC86-4CF27956C70A}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4" rowHeaderCaption="Department">
-  <location ref="A6:B9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9640BDDA-7F89-4B47-89C3-335567EC820D}" name="PivotTable3" cacheId="19" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Remote Work">
+  <location ref="A14:B17" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
-    <pivotField numFmtId="49" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item h="1" x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField dataField="1" showAll="0"/>
+    <pivotField dataField="1" numFmtId="49" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="3"/>
-  </rowFields>
-  <rowItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Average Salary" fld="4" subtotal="average" baseField="3" baseItem="0" numFmtId="43"/>
-  </dataFields>
-  <formats count="1">
-    <format dxfId="22">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="1">
-    <chartFormat chart="1" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotTable Style 1" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9640BDDA-7F89-4B47-89C3-335567EC820D}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Remote Work">
-  <location ref="A14:B17" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField dataField="1" numFmtId="49" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="1"/>
-        <item x="0"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
     <pivotField showAll="0"/>
     <pivotField axis="axisRow" showAll="0">
       <items count="4">
@@ -5442,7 +5425,7 @@
     <dataField name="Number of Employees" fld="0" subtotal="count" baseField="9" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="23">
+    <format dxfId="22">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -5493,21 +5476,14 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E06BAB96-9CD1-4BFF-B152-822D84770B56}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="City">
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E06BAB96-9CD1-4BFF-B152-822D84770B56}" name="PivotTable2" cacheId="19" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="City">
   <location ref="A23:B27" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField dataField="1" numFmtId="49" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
+    <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -5546,7 +5522,7 @@
     <dataField name="Number of Employees" fld="0" subtotal="count" baseField="7" baseItem="0" numFmtId="1"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="24">
+    <format dxfId="23">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -5573,9 +5549,82 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E9C9B4EC-AE72-4272-AC86-4CF27956C70A}" name="PivotTable1" cacheId="19" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4" rowHeaderCaption="Department">
+  <location ref="A6:B9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField numFmtId="49" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item h="1" x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Average Salary" fld="4" subtotal="average" baseField="3" baseItem="0" numFmtId="44"/>
+  </dataFields>
+  <formats count="2">
+    <format dxfId="25">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="24">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="1">
+    <chartFormat chart="1" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotTable Style 1" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{9BD59F20-4282-45EA-AB09-EBE730CAE810}" name="Table3" displayName="Table3" ref="O3:P6" totalsRowShown="0">
-  <autoFilter ref="O3:P6" xr:uid="{9BD59F20-4282-45EA-AB09-EBE730CAE810}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{9BD59F20-4282-45EA-AB09-EBE730CAE810}" name="Table3" displayName="Table3" ref="K3:L6" totalsRowShown="0">
+  <autoFilter ref="K3:L6" xr:uid="{9BD59F20-4282-45EA-AB09-EBE730CAE810}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{DE01E6C4-43F3-4B9A-92AA-6D293F1ECA62}" name="Issue Type"/>
     <tableColumn id="2" xr3:uid="{604F331C-F7B0-42F3-8B03-3E547CDB9108}" name="Count" dataDxfId="21"/>
@@ -5957,7 +6006,7 @@
   <sheetData>
     <row r="1" spans="1:1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="18.75" x14ac:dyDescent="0.3">
@@ -5965,32 +6014,32 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
@@ -6000,42 +6049,42 @@
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="15" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
@@ -6045,107 +6094,107 @@
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="28" spans="1:1" ht="45" x14ac:dyDescent="0.25">
       <c r="A28" s="13" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="39" spans="1:1" ht="45" x14ac:dyDescent="0.25">
       <c r="A39" s="13" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" s="8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
@@ -6155,62 +6204,62 @@
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" s="8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
@@ -6229,65 +6278,55 @@
   <sheetPr>
     <tabColor theme="9"/>
   </sheetPr>
-  <dimension ref="A1:P32"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr defaultColWidth="20.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="43.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="38.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="5.28515625" customWidth="1"/>
-    <col min="6" max="6" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="70.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.85546875" customWidth="1"/>
-    <col min="10" max="10" width="11.140625" customWidth="1"/>
-    <col min="11" max="11" width="10.140625" customWidth="1"/>
-    <col min="12" max="12" width="83.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="7.7109375" customWidth="1"/>
-    <col min="14" max="14" width="8.42578125" customWidth="1"/>
-    <col min="15" max="15" width="38" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12" customWidth="1"/>
+    <col min="6" max="6" width="129.28515625" customWidth="1"/>
+    <col min="8" max="8" width="70.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.7109375" customWidth="1"/>
+    <col min="10" max="10" width="8.42578125" customWidth="1"/>
+    <col min="11" max="11" width="21" customWidth="1"/>
+    <col min="12" max="12" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+    <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.25">
+      <c r="A1" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
-      <c r="L1" s="17"/>
-      <c r="M1" s="17"/>
-      <c r="N1" s="17"/>
-      <c r="O1" s="17"/>
-    </row>
-    <row r="2" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+    </row>
+    <row r="2" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="21" t="s">
+        <v>139</v>
+      </c>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="F2" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="F2" s="18" t="s">
+      <c r="G2" s="14"/>
+      <c r="H2" s="14" t="s">
         <v>141</v>
       </c>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
-      <c r="L2" s="14" t="s">
+      <c r="K2" s="22" t="s">
         <v>142</v>
       </c>
-      <c r="O2" s="19" t="s">
-        <v>143</v>
-      </c>
-      <c r="P2" s="19"/>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="L2" s="22"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>89</v>
       </c>
@@ -6296,99 +6335,99 @@
         <v>25</v>
       </c>
       <c r="C3" s="10"/>
+      <c r="H3" t="s">
+        <v>86</v>
+      </c>
+      <c r="K3" t="s">
+        <v>94</v>
+      </c>
       <c r="L3" t="s">
-        <v>86</v>
-      </c>
-      <c r="O3" t="s">
-        <v>94</v>
-      </c>
-      <c r="P3" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="L4" t="s">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H4" t="s">
         <v>87</v>
       </c>
-      <c r="O4" t="s">
+      <c r="K4" t="s">
         <v>96</v>
       </c>
-      <c r="P4" s="4">
+      <c r="L4" s="4">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="17">
         <f>AVERAGE('03_CLEANED_DATA'!E:E)</f>
         <v>79181.818181818177</v>
       </c>
       <c r="C5" s="9"/>
-      <c r="L5" t="s">
+      <c r="H5" t="s">
         <v>88</v>
       </c>
-      <c r="O5" t="s">
+      <c r="K5" t="s">
         <v>97</v>
       </c>
-      <c r="P5" s="4">
+      <c r="L5" s="4">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>3</v>
       </c>
       <c r="B6" t="s">
         <v>83</v>
       </c>
-      <c r="O6" t="s">
+      <c r="K6" t="s">
         <v>98</v>
       </c>
-      <c r="P6" s="4">
+      <c r="L6" s="4">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="16">
         <v>77200</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="16">
         <v>82700</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9" s="16">
         <v>79950</v>
       </c>
       <c r="C9" s="10"/>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B11" s="10">
         <f>AVERAGE('03_CLEANED_DATA'!F:F)</f>
         <v>7.8181818181818183</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="7"/>
       <c r="B12" s="5"/>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
         <v>91</v>
       </c>
@@ -6398,7 +6437,7 @@
       </c>
       <c r="C13" s="10"/>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>85</v>
       </c>
@@ -6406,7 +6445,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>77</v>
       </c>
@@ -6414,7 +6453,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
         <v>75</v>
       </c>
@@ -6422,7 +6461,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
         <v>80</v>
       </c>
@@ -6430,7 +6469,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
         <v>92</v>
       </c>
@@ -6440,12 +6479,12 @@
       </c>
       <c r="C20" s="11"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>7</v>
       </c>
@@ -6453,7 +6492,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
         <v>28</v>
       </c>
@@ -6461,41 +6500,44 @@
         <v>4</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B25" s="4">
         <v>16</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F25" s="8" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
         <v>30</v>
       </c>
       <c r="B26" s="4">
         <v>5</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F26" s="18" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
         <v>80</v>
       </c>
       <c r="B27" s="4">
         <v>25</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="G32" t="s">
-        <v>103</v>
+      <c r="F27" t="s">
+        <v>157</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:O1"/>
+  <mergeCells count="3">
+    <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:C2"/>
-    <mergeCell ref="F2:I2"/>
-    <mergeCell ref="O2:P2"/>
+    <mergeCell ref="K2:L2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId4"/>
@@ -6517,7 +6559,7 @@
     <col min="2" max="2" width="17.42578125" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="6.7109375" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.5703125" style="16" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="22.140625" style="4" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="20.85546875" style="4" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.5703125" style="3" bestFit="1" customWidth="1"/>
@@ -6538,7 +6580,7 @@
       <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="16" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="4" t="s">
@@ -6570,7 +6612,7 @@
       <c r="D2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="16">
         <v>75000</v>
       </c>
       <c r="F2" s="4">
@@ -6602,7 +6644,7 @@
       <c r="D3" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="16">
         <v>85000</v>
       </c>
       <c r="F3" s="4">
@@ -6631,7 +6673,7 @@
       <c r="D4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="16">
         <v>50000</v>
       </c>
       <c r="F4" s="4">
@@ -6660,7 +6702,7 @@
       <c r="D5" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="16">
         <v>120000</v>
       </c>
       <c r="F5" s="4">
@@ -6721,7 +6763,7 @@
       <c r="D7" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="16" t="s">
         <v>82</v>
       </c>
       <c r="F7" s="4">
@@ -6753,7 +6795,7 @@
       <c r="D8" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="16">
         <v>65000</v>
       </c>
       <c r="G8" s="4">
@@ -6782,7 +6824,7 @@
       <c r="D9" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="5">
+      <c r="E9" s="16">
         <v>70000</v>
       </c>
       <c r="F9" s="4">
@@ -6814,7 +6856,7 @@
       <c r="D10" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="16">
         <v>90000</v>
       </c>
       <c r="F10" s="4">
@@ -6846,7 +6888,7 @@
       <c r="D11" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E11" s="5">
+      <c r="E11" s="16">
         <v>95000</v>
       </c>
       <c r="F11" s="4">
@@ -6878,7 +6920,7 @@
       <c r="D12" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="16">
         <v>60000</v>
       </c>
       <c r="F12" s="4" t="s">
@@ -6910,7 +6952,7 @@
       <c r="D13" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E13" s="5">
+      <c r="E13" s="16">
         <v>88000</v>
       </c>
       <c r="F13" s="4">
@@ -6942,7 +6984,7 @@
       <c r="D14" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E14" s="5">
+      <c r="E14" s="16">
         <v>72000</v>
       </c>
       <c r="F14" s="4">
@@ -6974,7 +7016,7 @@
       <c r="D15" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="E15" s="5">
+      <c r="E15" s="16">
         <v>78000</v>
       </c>
       <c r="F15" s="4">
@@ -7006,7 +7048,7 @@
       <c r="D16" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E16" s="5">
+      <c r="E16" s="16">
         <v>110000</v>
       </c>
       <c r="F16" s="4" t="s">
@@ -7038,7 +7080,7 @@
       <c r="D17" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E17" s="5">
+      <c r="E17" s="16">
         <v>67000</v>
       </c>
       <c r="F17" s="4">
@@ -7070,7 +7112,7 @@
       <c r="D18" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E18" s="5" t="s">
+      <c r="E18" s="16" t="s">
         <v>82</v>
       </c>
       <c r="F18" s="4">
@@ -7102,7 +7144,7 @@
       <c r="D19" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E19" s="5">
+      <c r="E19" s="16">
         <v>82000</v>
       </c>
       <c r="F19" s="4">
@@ -7134,7 +7176,7 @@
       <c r="D20" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E20" s="5">
+      <c r="E20" s="16">
         <v>76000</v>
       </c>
       <c r="F20" s="4">
@@ -7166,7 +7208,7 @@
       <c r="D21" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E21" s="5">
+      <c r="E21" s="16">
         <v>92000</v>
       </c>
       <c r="F21" s="4">
@@ -7198,7 +7240,7 @@
       <c r="D22" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E22" s="5">
+      <c r="E22" s="16">
         <v>74000</v>
       </c>
       <c r="F22" s="4">
@@ -7230,7 +7272,7 @@
       <c r="D23" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E23" s="5">
+      <c r="E23" s="16">
         <v>86000</v>
       </c>
       <c r="F23" s="4">
@@ -7262,7 +7304,7 @@
       <c r="D24" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E24" s="5">
+      <c r="E24" s="16">
         <v>50000</v>
       </c>
       <c r="F24" s="4">
@@ -7294,7 +7336,7 @@
       <c r="D25" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E25" s="5">
+      <c r="E25" s="16">
         <v>73000</v>
       </c>
       <c r="F25" s="4">
@@ -7326,7 +7368,7 @@
       <c r="D26" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E26" s="5">
+      <c r="E26" s="16">
         <v>84000</v>
       </c>
       <c r="F26" s="4">

</xml_diff>